<commit_message>
Added Item Code column in all the material sample format xlsx sheets
</commit_message>
<xml_diff>
--- a/app/assets/data-import-samples/material/material_inward.xlsx
+++ b/app/assets/data-import-samples/material/material_inward.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
   <si>
     <t>Circle</t>
   </si>
@@ -57,6 +57,9 @@
   </si>
   <si>
     <t>DI No</t>
+  </si>
+  <si>
+    <t>Item Code</t>
   </si>
 </sst>
 </file>
@@ -413,22 +416,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="27.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="27.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>9</v>
       </c>
@@ -436,43 +440,47 @@
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="2"/>
+      <c r="H2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="2"/>
       <c r="I2" s="2"/>
-      <c r="J2" s="3" t="s">
+      <c r="J2" s="2"/>
+      <c r="K2" s="3" t="s">
         <v>7</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Development of Data Import
Added MRAD date column in material inward sample format file
</commit_message>
<xml_diff>
--- a/app/assets/data-import-samples/material/material_inward.xlsx
+++ b/app/assets/data-import-samples/material/material_inward.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="13">
   <si>
     <t>Circle</t>
   </si>
@@ -60,6 +60,9 @@
   </si>
   <si>
     <t>Item Code</t>
+  </si>
+  <si>
+    <t>MRAD Date</t>
   </si>
 </sst>
 </file>
@@ -416,7 +419,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
@@ -430,9 +433,10 @@
     <col min="9" max="9" width="11" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="17.5703125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="27.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>9</v>
       </c>
@@ -466,8 +470,11 @@
       <c r="K1" s="1" t="s">
         <v>8</v>
       </c>
+      <c r="L1" s="1" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -483,6 +490,9 @@
       <c r="K2" s="3" t="s">
         <v>7</v>
       </c>
+      <c r="L2" s="2" t="s">
+        <v>7</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>